<commit_message>
Update active officer registry
</commit_message>
<xml_diff>
--- a/public/assets/data/officers.xlsx
+++ b/public/assets/data/officers.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,49 +415,21 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>John Doe</v>
+        <v>Sesha Siva Sankar</v>
       </c>
       <c r="B2" t="str">
-        <v>john@unt.edu</v>
+        <v>SeshaSivaSankar@my.unt.edu</v>
       </c>
       <c r="C2" t="str">
-        <v>President</v>
+        <v>Super Admin</v>
       </c>
       <c r="D2" t="b">
         <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Jane Doe</v>
-      </c>
-      <c r="B3" t="str">
-        <v>jane@unt.edu</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Vice President</v>
-      </c>
-      <c r="D3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Former Officer</v>
-      </c>
-      <c r="B4" t="str">
-        <v>former@unt.edu</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Secretary</v>
-      </c>
-      <c r="D4" t="b">
-        <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>